<commit_message>
Se implementó reparación de formato de vuelos y horarios. Se aceptan guiones y espacios.
</commit_message>
<xml_diff>
--- a/Carga_Real.xlsx
+++ b/Carga_Real.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4043" uniqueCount="715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3996" uniqueCount="716">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -1487,7 +1487,7 @@
     <t xml:space="preserve">TK85 MNL IST</t>
   </si>
   <si>
-    <t xml:space="preserve">21:35 05:45+1</t>
+    <t xml:space="preserve">21:35-05:45+1</t>
   </si>
   <si>
     <t xml:space="preserve">TK801 IST PTY</t>
@@ -1496,10 +1496,13 @@
     <t xml:space="preserve">09:10-18:20</t>
   </si>
   <si>
+    <t xml:space="preserve">TK9608 PTY-SCL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:31 05:54+1</t>
+  </si>
+  <si>
     <t xml:space="preserve">TK9608 PTY - SCL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:31 05:54+1</t>
   </si>
   <si>
     <t xml:space="preserve">21:31-05:54+1</t>
@@ -3109,7 +3112,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="105" style="9" width="8.56"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -13608,7 +13611,7 @@
         <v>108</v>
       </c>
       <c r="D46" s="37" t="n">
-        <v>0</v>
+        <v>45322</v>
       </c>
       <c r="E46" s="37" t="n">
         <v>45612</v>
@@ -14574,13 +14577,13 @@
       <c r="AF50" s="39"/>
       <c r="AG50" s="36"/>
       <c r="AH50" s="36" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="AI50" s="37" t="n">
         <v>45610</v>
       </c>
       <c r="AJ50" s="37" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="AK50" s="52" t="s">
         <v>173</v>
@@ -15302,9 +15305,7 @@
       <c r="AG57" s="36"/>
       <c r="AH57" s="36"/>
       <c r="AI57" s="37"/>
-      <c r="AJ57" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ57" s="37"/>
       <c r="AK57" s="52"/>
       <c r="AL57" s="52"/>
       <c r="AM57" s="53"/>
@@ -15397,9 +15398,7 @@
       <c r="AG58" s="36"/>
       <c r="AH58" s="36"/>
       <c r="AI58" s="37"/>
-      <c r="AJ58" s="37" t="s">
-        <v>155</v>
-      </c>
+      <c r="AJ58" s="37"/>
       <c r="AK58" s="52"/>
       <c r="AL58" s="52"/>
       <c r="AM58" s="53"/>
@@ -15492,9 +15491,7 @@
       <c r="AG59" s="36"/>
       <c r="AH59" s="36"/>
       <c r="AI59" s="37"/>
-      <c r="AJ59" s="37" t="s">
-        <v>172</v>
-      </c>
+      <c r="AJ59" s="37"/>
       <c r="AK59" s="52"/>
       <c r="AL59" s="52"/>
       <c r="AM59" s="53"/>
@@ -15587,9 +15584,7 @@
       <c r="AG60" s="36"/>
       <c r="AH60" s="36"/>
       <c r="AI60" s="37"/>
-      <c r="AJ60" s="37" t="s">
-        <v>189</v>
-      </c>
+      <c r="AJ60" s="37"/>
       <c r="AK60" s="52"/>
       <c r="AL60" s="52"/>
       <c r="AM60" s="53"/>
@@ -15682,9 +15677,7 @@
       <c r="AG61" s="36"/>
       <c r="AH61" s="36"/>
       <c r="AI61" s="37"/>
-      <c r="AJ61" s="37" t="s">
-        <v>172</v>
-      </c>
+      <c r="AJ61" s="37"/>
       <c r="AK61" s="52"/>
       <c r="AL61" s="52"/>
       <c r="AM61" s="53"/>
@@ -15777,9 +15770,7 @@
       <c r="AG62" s="36"/>
       <c r="AH62" s="36"/>
       <c r="AI62" s="37"/>
-      <c r="AJ62" s="37" t="s">
-        <v>215</v>
-      </c>
+      <c r="AJ62" s="37"/>
       <c r="AK62" s="52"/>
       <c r="AL62" s="52"/>
       <c r="AM62" s="53"/>
@@ -15872,9 +15863,7 @@
       <c r="AG63" s="36"/>
       <c r="AH63" s="36"/>
       <c r="AI63" s="37"/>
-      <c r="AJ63" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ63" s="37"/>
       <c r="AK63" s="52"/>
       <c r="AL63" s="52"/>
       <c r="AM63" s="53"/>
@@ -15967,9 +15956,7 @@
       <c r="AG64" s="36"/>
       <c r="AH64" s="36"/>
       <c r="AI64" s="37"/>
-      <c r="AJ64" s="37" t="s">
-        <v>234</v>
-      </c>
+      <c r="AJ64" s="37"/>
       <c r="AK64" s="52"/>
       <c r="AL64" s="52"/>
       <c r="AM64" s="53"/>
@@ -16062,9 +16049,7 @@
       <c r="AG65" s="36"/>
       <c r="AH65" s="36"/>
       <c r="AI65" s="37"/>
-      <c r="AJ65" s="37" t="s">
-        <v>234</v>
-      </c>
+      <c r="AJ65" s="37"/>
       <c r="AK65" s="52"/>
       <c r="AL65" s="52"/>
       <c r="AM65" s="53"/>
@@ -16163,9 +16148,7 @@
       <c r="AG66" s="36"/>
       <c r="AH66" s="36"/>
       <c r="AI66" s="36"/>
-      <c r="AJ66" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ66" s="37"/>
       <c r="AK66" s="52"/>
       <c r="AL66" s="52"/>
       <c r="AM66" s="53"/>
@@ -16236,9 +16219,7 @@
       <c r="P67" s="1"/>
       <c r="Q67" s="3"/>
       <c r="X67" s="37"/>
-      <c r="AJ67" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ67" s="37"/>
       <c r="AK67" s="52"/>
       <c r="AL67" s="52"/>
       <c r="AM67" s="53"/>
@@ -16257,9 +16238,7 @@
       <c r="P68" s="1"/>
       <c r="Q68" s="3"/>
       <c r="X68" s="37"/>
-      <c r="AJ68" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ68" s="37"/>
       <c r="AK68" s="52"/>
       <c r="AL68" s="52"/>
       <c r="AM68" s="53"/>
@@ -16278,9 +16257,7 @@
       <c r="P69" s="1"/>
       <c r="Q69" s="3"/>
       <c r="X69" s="37"/>
-      <c r="AJ69" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ69" s="37"/>
       <c r="AK69" s="52"/>
       <c r="AL69" s="52"/>
       <c r="AM69" s="53"/>
@@ -16299,9 +16276,7 @@
       <c r="P70" s="1"/>
       <c r="Q70" s="3"/>
       <c r="X70" s="37"/>
-      <c r="AJ70" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ70" s="37"/>
       <c r="AK70" s="52"/>
       <c r="AL70" s="52"/>
       <c r="AM70" s="53"/>
@@ -16320,9 +16295,7 @@
       <c r="P71" s="1"/>
       <c r="Q71" s="3"/>
       <c r="X71" s="37"/>
-      <c r="AJ71" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ71" s="37"/>
       <c r="AK71" s="52"/>
       <c r="AL71" s="52"/>
       <c r="AM71" s="53"/>
@@ -16341,9 +16314,7 @@
       <c r="P72" s="1"/>
       <c r="Q72" s="3"/>
       <c r="X72" s="37"/>
-      <c r="AJ72" s="37" t="s">
-        <v>172</v>
-      </c>
+      <c r="AJ72" s="37"/>
       <c r="AK72" s="52"/>
       <c r="AL72" s="52"/>
       <c r="AM72" s="53"/>
@@ -16362,9 +16333,7 @@
       <c r="P73" s="1"/>
       <c r="Q73" s="3"/>
       <c r="X73" s="37"/>
-      <c r="AJ73" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ73" s="37"/>
       <c r="AK73" s="52"/>
       <c r="AL73" s="52"/>
       <c r="AM73" s="53"/>
@@ -16383,9 +16352,7 @@
       <c r="P74" s="1"/>
       <c r="Q74" s="3"/>
       <c r="X74" s="37"/>
-      <c r="AJ74" s="37" t="s">
-        <v>127</v>
-      </c>
+      <c r="AJ74" s="37"/>
       <c r="AK74" s="52"/>
       <c r="AL74" s="52"/>
       <c r="AM74" s="53"/>
@@ -16404,9 +16371,7 @@
       <c r="P75" s="1"/>
       <c r="Q75" s="3"/>
       <c r="X75" s="37"/>
-      <c r="AJ75" s="37" t="s">
-        <v>234</v>
-      </c>
+      <c r="AJ75" s="37"/>
       <c r="AK75" s="52"/>
       <c r="AL75" s="52"/>
       <c r="AM75" s="53"/>
@@ -16425,9 +16390,7 @@
       <c r="P76" s="1"/>
       <c r="Q76" s="3"/>
       <c r="X76" s="37"/>
-      <c r="AJ76" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ76" s="37"/>
       <c r="AK76" s="52"/>
       <c r="AL76" s="52"/>
       <c r="AM76" s="53"/>
@@ -16446,9 +16409,7 @@
       <c r="P77" s="1"/>
       <c r="Q77" s="3"/>
       <c r="X77" s="37"/>
-      <c r="AJ77" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ77" s="37"/>
       <c r="AK77" s="52"/>
       <c r="AL77" s="52"/>
       <c r="AM77" s="53"/>
@@ -16467,9 +16428,7 @@
       <c r="P78" s="1"/>
       <c r="Q78" s="3"/>
       <c r="X78" s="37"/>
-      <c r="AJ78" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ78" s="37"/>
       <c r="AK78" s="52"/>
       <c r="AL78" s="52"/>
       <c r="AM78" s="53"/>
@@ -16488,9 +16447,7 @@
       <c r="P79" s="1"/>
       <c r="Q79" s="3"/>
       <c r="X79" s="37"/>
-      <c r="AJ79" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ79" s="37"/>
       <c r="AK79" s="52"/>
       <c r="AL79" s="52"/>
       <c r="AM79" s="53"/>
@@ -16509,9 +16466,7 @@
       <c r="P80" s="1"/>
       <c r="Q80" s="3"/>
       <c r="X80" s="37"/>
-      <c r="AJ80" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ80" s="37"/>
       <c r="AK80" s="56"/>
       <c r="AL80" s="56"/>
       <c r="AM80" s="57"/>
@@ -16530,9 +16485,7 @@
       <c r="P81" s="1"/>
       <c r="Q81" s="3"/>
       <c r="X81" s="37"/>
-      <c r="AJ81" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ81" s="37"/>
       <c r="AK81" s="52"/>
       <c r="AL81" s="52"/>
       <c r="AM81" s="53"/>
@@ -16551,9 +16504,7 @@
       <c r="P82" s="1"/>
       <c r="Q82" s="3"/>
       <c r="X82" s="37"/>
-      <c r="AJ82" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ82" s="37"/>
       <c r="AK82" s="52"/>
       <c r="AL82" s="52"/>
       <c r="AM82" s="53"/>
@@ -16572,9 +16523,7 @@
       <c r="P83" s="1"/>
       <c r="Q83" s="3"/>
       <c r="X83" s="37"/>
-      <c r="AJ83" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ83" s="37"/>
       <c r="AK83" s="56"/>
       <c r="AL83" s="56"/>
       <c r="AM83" s="57"/>
@@ -16593,9 +16542,7 @@
       <c r="P84" s="1"/>
       <c r="Q84" s="3"/>
       <c r="X84" s="37"/>
-      <c r="AJ84" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ84" s="37"/>
       <c r="AK84" s="52"/>
       <c r="AL84" s="52"/>
       <c r="AM84" s="53"/>
@@ -16614,9 +16561,7 @@
       <c r="P85" s="1"/>
       <c r="Q85" s="3"/>
       <c r="X85" s="37"/>
-      <c r="AJ85" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ85" s="37"/>
       <c r="AK85" s="56"/>
       <c r="AL85" s="56"/>
       <c r="AM85" s="57"/>
@@ -16634,9 +16579,7 @@
       <c r="P86" s="1"/>
       <c r="Q86" s="3"/>
       <c r="X86" s="37"/>
-      <c r="AJ86" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ86" s="37"/>
       <c r="AK86" s="52"/>
       <c r="AL86" s="52"/>
       <c r="AM86" s="53"/>
@@ -16654,9 +16597,7 @@
       <c r="P87" s="1"/>
       <c r="Q87" s="3"/>
       <c r="X87" s="37"/>
-      <c r="AJ87" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ87" s="37"/>
       <c r="AK87" s="52"/>
       <c r="AL87" s="52"/>
       <c r="AM87" s="53"/>
@@ -16674,9 +16615,7 @@
       <c r="P88" s="1"/>
       <c r="Q88" s="3"/>
       <c r="X88" s="37"/>
-      <c r="AJ88" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ88" s="37"/>
       <c r="AK88" s="52"/>
       <c r="AL88" s="52"/>
       <c r="AM88" s="53"/>
@@ -16694,9 +16633,7 @@
       <c r="P89" s="1"/>
       <c r="Q89" s="3"/>
       <c r="X89" s="37"/>
-      <c r="AJ89" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ89" s="37"/>
       <c r="AK89" s="52"/>
       <c r="AL89" s="52"/>
       <c r="AM89" s="53"/>
@@ -16714,9 +16651,7 @@
       <c r="P90" s="1"/>
       <c r="Q90" s="3"/>
       <c r="X90" s="37"/>
-      <c r="AJ90" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ90" s="37"/>
       <c r="AK90" s="52"/>
       <c r="AL90" s="52"/>
       <c r="AM90" s="53"/>
@@ -16734,9 +16669,7 @@
       <c r="P91" s="1"/>
       <c r="Q91" s="3"/>
       <c r="X91" s="37"/>
-      <c r="AJ91" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ91" s="37"/>
       <c r="AK91" s="52"/>
       <c r="AL91" s="52"/>
       <c r="AM91" s="53"/>
@@ -16754,9 +16687,7 @@
       <c r="P92" s="1"/>
       <c r="Q92" s="3"/>
       <c r="X92" s="37"/>
-      <c r="AJ92" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ92" s="37"/>
       <c r="AK92" s="52"/>
       <c r="AL92" s="52"/>
       <c r="AM92" s="53"/>
@@ -16774,9 +16705,7 @@
       <c r="P93" s="1"/>
       <c r="Q93" s="3"/>
       <c r="X93" s="37"/>
-      <c r="AJ93" s="37" t="s">
-        <v>234</v>
-      </c>
+      <c r="AJ93" s="37"/>
       <c r="AK93" s="52"/>
       <c r="AL93" s="52"/>
       <c r="AM93" s="53"/>
@@ -16792,9 +16721,7 @@
       <c r="P94" s="1"/>
       <c r="Q94" s="3"/>
       <c r="X94" s="37"/>
-      <c r="AJ94" s="37" t="s">
-        <v>413</v>
-      </c>
+      <c r="AJ94" s="37"/>
       <c r="AK94" s="52"/>
       <c r="AL94" s="52"/>
       <c r="AM94" s="53"/>
@@ -16810,9 +16737,7 @@
       <c r="P95" s="1"/>
       <c r="Q95" s="3"/>
       <c r="X95" s="37"/>
-      <c r="AJ95" s="37" t="s">
-        <v>215</v>
-      </c>
+      <c r="AJ95" s="37"/>
       <c r="AK95" s="52"/>
       <c r="AL95" s="52"/>
       <c r="AM95" s="53"/>
@@ -16828,9 +16753,7 @@
       <c r="P96" s="1"/>
       <c r="Q96" s="3"/>
       <c r="X96" s="37"/>
-      <c r="AJ96" s="37" t="s">
-        <v>435</v>
-      </c>
+      <c r="AJ96" s="37"/>
       <c r="AK96" s="52"/>
       <c r="AL96" s="52"/>
       <c r="AM96" s="53"/>
@@ -16846,9 +16769,7 @@
       <c r="P97" s="1"/>
       <c r="Q97" s="3"/>
       <c r="X97" s="37"/>
-      <c r="AJ97" s="37" t="s">
-        <v>444</v>
-      </c>
+      <c r="AJ97" s="37"/>
       <c r="AK97" s="52"/>
       <c r="AL97" s="52"/>
       <c r="AM97" s="53"/>
@@ -16864,9 +16785,7 @@
       <c r="P98" s="1"/>
       <c r="Q98" s="3"/>
       <c r="X98" s="37"/>
-      <c r="AJ98" s="37" t="s">
-        <v>444</v>
-      </c>
+      <c r="AJ98" s="37"/>
       <c r="AK98" s="52"/>
       <c r="AL98" s="52"/>
       <c r="AM98" s="53"/>
@@ -16882,9 +16801,7 @@
       <c r="P99" s="1"/>
       <c r="Q99" s="3"/>
       <c r="X99" s="37"/>
-      <c r="AJ99" s="37" t="s">
-        <v>318</v>
-      </c>
+      <c r="AJ99" s="37"/>
       <c r="AK99" s="56"/>
       <c r="AL99" s="56"/>
       <c r="AM99" s="57"/>
@@ -16900,9 +16817,7 @@
       <c r="P100" s="1"/>
       <c r="Q100" s="3"/>
       <c r="X100" s="37"/>
-      <c r="AJ100" s="37" t="s">
-        <v>444</v>
-      </c>
+      <c r="AJ100" s="37"/>
       <c r="AK100" s="52"/>
       <c r="AL100" s="52"/>
       <c r="AM100" s="53"/>
@@ -16934,9 +16849,7 @@
       <c r="P102" s="1"/>
       <c r="Q102" s="3"/>
       <c r="X102" s="37"/>
-      <c r="AJ102" s="37" t="s">
-        <v>172</v>
-      </c>
+      <c r="AJ102" s="37"/>
       <c r="AK102" s="52"/>
       <c r="AL102" s="52"/>
       <c r="AM102" s="53"/>
@@ -16952,9 +16865,7 @@
       <c r="P103" s="1"/>
       <c r="Q103" s="3"/>
       <c r="X103" s="37"/>
-      <c r="AJ103" s="37" t="s">
-        <v>435</v>
-      </c>
+      <c r="AJ103" s="37"/>
       <c r="AK103" s="52"/>
       <c r="AL103" s="52"/>
       <c r="AM103" s="53"/>
@@ -16986,9 +16897,7 @@
       <c r="P105" s="1"/>
       <c r="Q105" s="3"/>
       <c r="X105" s="37"/>
-      <c r="AJ105" s="37" t="s">
-        <v>492</v>
-      </c>
+      <c r="AJ105" s="37"/>
       <c r="AK105" s="52"/>
       <c r="AL105" s="52"/>
       <c r="AM105" s="53"/>
@@ -17004,10 +16913,7 @@
       <c r="P106" s="1"/>
       <c r="Q106" s="3"/>
       <c r="X106" s="37"/>
-      <c r="AJ106" s="37" t="str">
-        <f aca="false">TRIM(AJ51)</f>
-        <v/>
-      </c>
+      <c r="AJ106" s="37"/>
       <c r="AK106" s="52"/>
       <c r="AL106" s="52"/>
       <c r="AM106" s="53"/>
@@ -17017,7 +16923,7 @@
       <c r="AU106" s="36"/>
       <c r="AV106" s="36"/>
     </row>
-    <row r="107" customFormat="false" ht="10.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="10.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E107" s="62"/>
       <c r="M107" s="9"/>
       <c r="P107" s="1"/>
@@ -17032,7 +16938,7 @@
       <c r="AU107" s="36"/>
       <c r="AV107" s="36"/>
     </row>
-    <row r="108" customFormat="false" ht="10.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="10.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E108" s="62"/>
       <c r="M108" s="9"/>
       <c r="P108" s="1"/>
@@ -17047,7 +16953,7 @@
       <c r="AU108" s="36"/>
       <c r="AV108" s="36"/>
     </row>
-    <row r="109" customFormat="false" ht="10.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="10.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E109" s="62"/>
       <c r="M109" s="9"/>
       <c r="P109" s="1"/>
@@ -18120,13 +18026,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="12.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="8.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="8.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11"/>
@@ -18221,7 +18127,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="68" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E1" s="68" t="s">
         <v>4</v>
@@ -18230,13 +18136,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>9</v>
@@ -18523,25 +18429,25 @@
         <v>145</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>114</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="P2" s="9" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="Q2" s="77" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="R2" s="9" t="s">
         <v>120</v>
@@ -18556,19 +18462,19 @@
         <v>120</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="W2" s="4"/>
       <c r="Z2" s="8"/>
       <c r="AA2" s="78"/>
       <c r="AB2" s="78" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="AC2" s="8" t="n">
         <v>45613</v>
       </c>
       <c r="AD2" s="79" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="AE2" s="78"/>
       <c r="AF2" s="38"/>
@@ -18580,7 +18486,7 @@
       <c r="AR2" s="4"/>
       <c r="AS2" s="4"/>
       <c r="AV2" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="AW2" s="4" t="n">
         <v>45612</v>
@@ -18592,7 +18498,7 @@
         <v>192</v>
       </c>
       <c r="AZ2" s="9" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="BA2" s="36"/>
       <c r="BB2" s="36"/>
@@ -18618,7 +18524,7 @@
       <c r="BW2" s="37"/>
       <c r="BX2" s="80"/>
       <c r="BY2" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="CO2" s="4"/>
     </row>
@@ -18651,77 +18557,77 @@
         <v>145</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>114</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="O3" s="9" t="s">
         <v>391</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="Q3" s="77" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S3" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T3" s="9" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="V3" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W3" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X3" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="Z3" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA3" s="78" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB3" s="78" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="AC3" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD3" s="79" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="AE3" s="78"/>
       <c r="AF3" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH3" s="38" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ3" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AL3" s="36" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM3" s="8" t="n">
         <v>45612</v>
@@ -18730,10 +18636,10 @@
         <v>45614</v>
       </c>
       <c r="AO3" s="9" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="AP3" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ3" s="9" t="s">
         <v>135</v>
@@ -18745,7 +18651,7 @@
         <v>45615</v>
       </c>
       <c r="AT3" s="9" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="AU3" s="9" t="s">
         <v>176</v>
@@ -18823,10 +18729,10 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY3" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ3" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA3" s="67" t="n">
         <v>45612</v>
@@ -18835,10 +18741,10 @@
         <v>45613</v>
       </c>
       <c r="CC3" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD3" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE3" s="67" t="n">
         <v>45612</v>
@@ -18847,7 +18753,7 @@
         <v>45613</v>
       </c>
       <c r="CG3" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18879,10 +18785,10 @@
         <v>145</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>148</v>
@@ -18891,13 +18797,13 @@
         <v>480</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="Q4" s="77" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="R4" s="9" t="s">
         <v>120</v>
@@ -18982,10 +18888,10 @@
         <v>145</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>148</v>
@@ -18997,10 +18903,10 @@
         <v>163</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="Q5" s="77" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="R5" s="9" t="s">
         <v>120</v>
@@ -19015,7 +18921,7 @@
         <v>120</v>
       </c>
       <c r="V5" s="9" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="W5" s="8" t="n">
         <v>45612</v>
@@ -19023,23 +18929,23 @@
       <c r="Z5" s="8"/>
       <c r="AA5" s="78"/>
       <c r="AB5" s="78" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="AC5" s="8" t="n">
         <v>45613</v>
       </c>
       <c r="AD5" s="79" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="AE5" s="78"/>
       <c r="AF5" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH5" s="38" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ5" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK5" s="2"/>
       <c r="AL5" s="1"/>
@@ -19048,7 +18954,7 @@
       <c r="AR5" s="8"/>
       <c r="AS5" s="8"/>
       <c r="AV5" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="AW5" s="8" t="n">
         <v>45612</v>
@@ -19060,7 +18966,7 @@
         <v>175</v>
       </c>
       <c r="AZ5" s="9" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="BA5" s="36"/>
       <c r="BB5" s="36"/>
@@ -19116,10 +19022,10 @@
         <v>145</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>148</v>
@@ -19131,65 +19037,65 @@
         <v>238</v>
       </c>
       <c r="P6" s="9" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="Q6" s="77" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S6" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T6" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U6" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V6" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W6" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X6" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="Z6" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA6" s="78" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AB6" s="78" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC6" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD6" s="79" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE6" s="78"/>
       <c r="AF6" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH6" s="38" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ6" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL6" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM6" s="8" t="n">
         <v>45612</v>
@@ -19201,7 +19107,7 @@
         <v>158</v>
       </c>
       <c r="AP6" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ6" s="9" t="s">
         <v>135</v>
@@ -19216,7 +19122,7 @@
         <v>158</v>
       </c>
       <c r="AU6" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW6" s="8"/>
       <c r="AX6" s="8"/>
@@ -19291,7 +19197,7 @@
         <v>0.0215277777777778</v>
       </c>
       <c r="BY6" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ6" s="9" t="s">
         <v>143</v>
@@ -19303,7 +19209,7 @@
         <v>45614</v>
       </c>
       <c r="CC6" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD6" s="9" t="s">
         <v>144</v>
@@ -19344,10 +19250,10 @@
         <v>145</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>148</v>
@@ -19359,65 +19265,65 @@
         <v>218</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="Q7" s="77" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S7" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T7" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U7" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V7" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W7" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X7" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z7" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA7" s="78" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB7" s="78" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC7" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD7" s="79" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE7" s="78"/>
       <c r="AF7" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH7" s="38" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ7" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL7" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM7" s="8" t="n">
         <v>45612</v>
@@ -19429,7 +19335,7 @@
         <v>158</v>
       </c>
       <c r="AP7" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ7" s="9" t="s">
         <v>135</v>
@@ -19444,7 +19350,7 @@
         <v>158</v>
       </c>
       <c r="AU7" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW7" s="8"/>
       <c r="AX7" s="8"/>
@@ -19519,7 +19425,7 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY7" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ7" s="9" t="s">
         <v>143</v>
@@ -19531,7 +19437,7 @@
         <v>45614</v>
       </c>
       <c r="CC7" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD7" s="9" t="s">
         <v>144</v>
@@ -19573,10 +19479,10 @@
         <v>145</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>148</v>
@@ -19588,65 +19494,65 @@
         <v>238</v>
       </c>
       <c r="P8" s="9" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="Q8" s="77" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="R8" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S8" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T8" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U8" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V8" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W8" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X8" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z8" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA8" s="78" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB8" s="78" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC8" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD8" s="79" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE8" s="78"/>
       <c r="AF8" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH8" s="38" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ8" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL8" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM8" s="8" t="n">
         <v>45612</v>
@@ -19658,7 +19564,7 @@
         <v>158</v>
       </c>
       <c r="AP8" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ8" s="9" t="s">
         <v>135</v>
@@ -19673,7 +19579,7 @@
         <v>158</v>
       </c>
       <c r="AU8" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW8" s="8"/>
       <c r="AX8" s="8"/>
@@ -19748,7 +19654,7 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY8" s="1" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="BZ8" s="9" t="s">
         <v>143</v>
@@ -19760,7 +19666,7 @@
         <v>45614</v>
       </c>
       <c r="CC8" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD8" s="9" t="s">
         <v>144</v>
@@ -19801,10 +19707,10 @@
         <v>145</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>148</v>
@@ -19816,65 +19722,65 @@
         <v>238</v>
       </c>
       <c r="P9" s="9" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="Q9" s="77" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="R9" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S9" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T9" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U9" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V9" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W9" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X9" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y9" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z9" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA9" s="78" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB9" s="78" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC9" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD9" s="79" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE9" s="78"/>
       <c r="AF9" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH9" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ9" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK9" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL9" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM9" s="8" t="n">
         <v>45612</v>
@@ -19886,7 +19792,7 @@
         <v>158</v>
       </c>
       <c r="AP9" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ9" s="9" t="s">
         <v>135</v>
@@ -19901,7 +19807,7 @@
         <v>158</v>
       </c>
       <c r="AU9" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW9" s="8"/>
       <c r="AX9" s="8"/>
@@ -19976,7 +19882,7 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY9" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ9" s="9" t="s">
         <v>143</v>
@@ -19988,7 +19894,7 @@
         <v>45614</v>
       </c>
       <c r="CC9" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD9" s="9" t="s">
         <v>144</v>
@@ -20029,10 +19935,10 @@
         <v>145</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>148</v>
@@ -20044,65 +19950,65 @@
         <v>255</v>
       </c>
       <c r="P10" s="9" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="Q10" s="77" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S10" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T10" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U10" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V10" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W10" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X10" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z10" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA10" s="78" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="AB10" s="78" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC10" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD10" s="79" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE10" s="78"/>
       <c r="AF10" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH10" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ10" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL10" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM10" s="8" t="n">
         <v>45612</v>
@@ -20114,7 +20020,7 @@
         <v>158</v>
       </c>
       <c r="AP10" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ10" s="9" t="s">
         <v>135</v>
@@ -20129,7 +20035,7 @@
         <v>158</v>
       </c>
       <c r="AU10" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW10" s="8"/>
       <c r="AX10" s="8"/>
@@ -20204,7 +20110,7 @@
         <v>0.0472222222222222</v>
       </c>
       <c r="BY10" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ10" s="9" t="s">
         <v>144</v>
@@ -20216,7 +20122,7 @@
         <v>45616</v>
       </c>
       <c r="CC10" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20248,10 +20154,10 @@
         <v>145</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>148</v>
@@ -20263,64 +20169,64 @@
         <v>267</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="Q11" s="77" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="R11" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S11" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T11" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U11" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V11" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W11" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X11" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y11" s="5" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="Z11" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA11" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AB11" s="9" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC11" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD11" s="65" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AF11" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH11" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ11" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK11" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL11" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM11" s="8" t="n">
         <v>45612</v>
@@ -20332,7 +20238,7 @@
         <v>175</v>
       </c>
       <c r="AP11" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ11" s="9" t="s">
         <v>135</v>
@@ -20347,7 +20253,7 @@
         <v>175</v>
       </c>
       <c r="AU11" s="9" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="AW11" s="8"/>
       <c r="AX11" s="8"/>
@@ -20422,10 +20328,10 @@
         <v>0.0215277777777778</v>
       </c>
       <c r="BY11" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ11" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA11" s="67" t="n">
         <v>45612</v>
@@ -20434,10 +20340,10 @@
         <v>45613</v>
       </c>
       <c r="CC11" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD11" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE11" s="67" t="n">
         <v>45612</v>
@@ -20446,7 +20352,7 @@
         <v>45613</v>
       </c>
       <c r="CG11" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20478,10 +20384,10 @@
         <v>145</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>114</v>
@@ -20493,64 +20399,64 @@
         <v>238</v>
       </c>
       <c r="P12" s="9" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="Q12" s="77" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="R12" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S12" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T12" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U12" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V12" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W12" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X12" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y12" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z12" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA12" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB12" s="9" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC12" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD12" s="65" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AF12" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH12" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ12" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK12" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL12" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM12" s="8" t="n">
         <v>45612</v>
@@ -20562,7 +20468,7 @@
         <v>136</v>
       </c>
       <c r="AP12" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ12" s="9" t="s">
         <v>135</v>
@@ -20577,7 +20483,7 @@
         <v>136</v>
       </c>
       <c r="AU12" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW12" s="8"/>
       <c r="AX12" s="8"/>
@@ -20652,10 +20558,10 @@
         <v>0.0284722222222222</v>
       </c>
       <c r="BY12" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ12" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA12" s="67" t="n">
         <v>45612</v>
@@ -20664,10 +20570,10 @@
         <v>45613</v>
       </c>
       <c r="CC12" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD12" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE12" s="67" t="n">
         <v>45612</v>
@@ -20676,7 +20582,7 @@
         <v>45613</v>
       </c>
       <c r="CG12" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20708,10 +20614,10 @@
         <v>145</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>148</v>
@@ -20723,64 +20629,64 @@
         <v>329</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="Q13" s="77" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="R13" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S13" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T13" s="9" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="U13" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V13" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W13" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X13" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y13" s="5" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="Z13" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA13" s="9" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="AB13" s="9" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="AC13" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD13" s="65" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="AF13" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH13" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ13" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK13" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL13" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM13" s="8" t="n">
         <v>45612</v>
@@ -20792,7 +20698,7 @@
         <v>158</v>
       </c>
       <c r="AP13" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ13" s="9" t="s">
         <v>135</v>
@@ -20807,7 +20713,7 @@
         <v>158</v>
       </c>
       <c r="AU13" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW13" s="8"/>
       <c r="AX13" s="8"/>
@@ -20882,10 +20788,10 @@
         <v>0.328472222222222</v>
       </c>
       <c r="BY13" s="1" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="BZ13" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA13" s="67" t="n">
         <v>45612</v>
@@ -20894,10 +20800,10 @@
         <v>45613</v>
       </c>
       <c r="CC13" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD13" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE13" s="67" t="n">
         <v>45612</v>
@@ -20906,7 +20812,7 @@
         <v>45613</v>
       </c>
       <c r="CG13" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20938,10 +20844,10 @@
         <v>145</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>148</v>
@@ -20953,13 +20859,13 @@
         <v>209</v>
       </c>
       <c r="P14" s="9" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="Q14" s="77" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="R14" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S14" s="9" t="s">
         <v>119</v>
@@ -20971,46 +20877,46 @@
         <v>120</v>
       </c>
       <c r="V14" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W14" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X14" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y14" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z14" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA14" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB14" s="9" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="AC14" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD14" s="65" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="AF14" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH14" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ14" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK14" s="2" t="n">
         <v>2</v>
       </c>
       <c r="AL14" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM14" s="8" t="n">
         <v>45612</v>
@@ -21022,7 +20928,7 @@
         <v>158</v>
       </c>
       <c r="AP14" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ14" s="9" t="s">
         <v>135</v>
@@ -21037,7 +20943,7 @@
         <v>158</v>
       </c>
       <c r="AU14" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW14" s="8"/>
       <c r="AX14" s="8"/>
@@ -21112,10 +21018,10 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY14" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ14" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA14" s="67" t="n">
         <v>45612</v>
@@ -21124,10 +21030,10 @@
         <v>45613</v>
       </c>
       <c r="CC14" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD14" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE14" s="67" t="n">
         <v>45612</v>
@@ -21136,7 +21042,7 @@
         <v>45613</v>
       </c>
       <c r="CG14" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21168,10 +21074,10 @@
         <v>145</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>148</v>
@@ -21183,13 +21089,13 @@
         <v>329</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="Q15" s="77" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="R15" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S15" s="9" t="s">
         <v>119</v>
@@ -21201,46 +21107,46 @@
         <v>120</v>
       </c>
       <c r="V15" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W15" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X15" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y15" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z15" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA15" s="9" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="AB15" s="9" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="AC15" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD15" s="65" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="AF15" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH15" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ15" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AL15" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM15" s="8" t="n">
         <v>45612</v>
@@ -21252,7 +21158,7 @@
         <v>158</v>
       </c>
       <c r="AP15" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ15" s="9" t="s">
         <v>135</v>
@@ -21267,7 +21173,7 @@
         <v>158</v>
       </c>
       <c r="AU15" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW15" s="8"/>
       <c r="AX15" s="8"/>
@@ -21342,7 +21248,7 @@
         <v>0.0472222222222222</v>
       </c>
       <c r="BY15" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ15" s="9" t="s">
         <v>144</v>
@@ -21354,7 +21260,7 @@
         <v>45616</v>
       </c>
       <c r="CC15" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21386,10 +21292,10 @@
         <v>145</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>148</v>
@@ -21401,13 +21307,13 @@
         <v>262</v>
       </c>
       <c r="P16" s="9" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="Q16" s="77" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="R16" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S16" s="9" t="s">
         <v>119</v>
@@ -21419,46 +21325,46 @@
         <v>120</v>
       </c>
       <c r="V16" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W16" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X16" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y16" s="5" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="Z16" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA16" s="9" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="AB16" s="9" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="AC16" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD16" s="65" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="AF16" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH16" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ16" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL16" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM16" s="8" t="n">
         <v>45612</v>
@@ -21470,12 +21376,12 @@
         <v>158</v>
       </c>
       <c r="AP16" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AR16" s="8"/>
       <c r="AS16" s="8"/>
       <c r="AV16" s="9" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="AW16" s="8" t="n">
         <v>45615</v>
@@ -21487,7 +21393,7 @@
         <v>158</v>
       </c>
       <c r="AZ16" s="9" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="BA16" s="1" t="s">
         <v>141</v>
@@ -21565,10 +21471,10 @@
         <v>145</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="M17" s="1" t="s">
         <v>148</v>
@@ -21580,13 +21486,13 @@
         <v>404</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="Q17" s="77" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S17" s="9" t="s">
         <v>119</v>
@@ -21598,46 +21504,46 @@
         <v>120</v>
       </c>
       <c r="V17" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W17" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X17" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y17" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z17" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA17" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB17" s="9" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="AC17" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD17" s="65" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="AF17" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH17" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ17" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK17" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL17" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM17" s="8" t="n">
         <v>45612</v>
@@ -21649,7 +21555,7 @@
         <v>158</v>
       </c>
       <c r="AP17" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ17" s="9" t="s">
         <v>135</v>
@@ -21664,7 +21570,7 @@
         <v>158</v>
       </c>
       <c r="AU17" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AW17" s="8"/>
       <c r="AX17" s="8"/>
@@ -21739,10 +21645,10 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY17" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ17" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA17" s="67" t="n">
         <v>45612</v>
@@ -21751,10 +21657,10 @@
         <v>45613</v>
       </c>
       <c r="CC17" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD17" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE17" s="67" t="n">
         <v>45612</v>
@@ -21763,7 +21669,7 @@
         <v>45613</v>
       </c>
       <c r="CG17" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21795,28 +21701,28 @@
         <v>145</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>114</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="O18" s="9" t="s">
         <v>116</v>
       </c>
       <c r="P18" s="9" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="Q18" s="77" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="R18" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S18" s="9" t="s">
         <v>119</v>
@@ -21828,46 +21734,46 @@
         <v>120</v>
       </c>
       <c r="V18" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W18" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X18" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y18" s="5" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="Z18" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA18" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AB18" s="9" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="AC18" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD18" s="65" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="AF18" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH18" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ18" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL18" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM18" s="8" t="n">
         <v>45612</v>
@@ -21879,7 +21785,7 @@
         <v>136</v>
       </c>
       <c r="AP18" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ18" s="9" t="s">
         <v>135</v>
@@ -21894,7 +21800,7 @@
         <v>136</v>
       </c>
       <c r="AU18" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA18" s="1" t="s">
         <v>141</v>
@@ -21967,10 +21873,10 @@
         <v>0.0215277777777778</v>
       </c>
       <c r="BY18" s="1" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="BZ18" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA18" s="67" t="n">
         <v>45612</v>
@@ -21979,10 +21885,10 @@
         <v>45613</v>
       </c>
       <c r="CC18" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD18" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE18" s="67" t="n">
         <v>45612</v>
@@ -21991,7 +21897,7 @@
         <v>45613</v>
       </c>
       <c r="CG18" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22023,28 +21929,28 @@
         <v>145</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>148</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>348</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="Q19" s="77" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="R19" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S19" s="9" t="s">
         <v>119</v>
@@ -22056,46 +21962,46 @@
         <v>120</v>
       </c>
       <c r="V19" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W19" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X19" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y19" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z19" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA19" s="9" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="AB19" s="9" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="AC19" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD19" s="65" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="AF19" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH19" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ19" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK19" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL19" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM19" s="8" t="n">
         <v>45612</v>
@@ -22107,7 +22013,7 @@
         <v>175</v>
       </c>
       <c r="AP19" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ19" s="9" t="s">
         <v>135</v>
@@ -22122,7 +22028,7 @@
         <v>175</v>
       </c>
       <c r="AU19" s="9" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="BA19" s="1" t="s">
         <v>141</v>
@@ -22195,10 +22101,10 @@
         <v>0.915972222222222</v>
       </c>
       <c r="BY19" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ19" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA19" s="67" t="n">
         <v>45612</v>
@@ -22207,10 +22113,10 @@
         <v>45613</v>
       </c>
       <c r="CC19" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD19" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE19" s="67" t="n">
         <v>45612</v>
@@ -22219,7 +22125,7 @@
         <v>45613</v>
       </c>
       <c r="CG19" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22251,10 +22157,10 @@
         <v>145</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="M20" s="1" t="s">
         <v>148</v>
@@ -22266,13 +22172,13 @@
         <v>372</v>
       </c>
       <c r="P20" s="9" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="Q20" s="77" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="R20" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S20" s="9" t="s">
         <v>119</v>
@@ -22284,46 +22190,46 @@
         <v>120</v>
       </c>
       <c r="V20" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W20" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X20" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y20" s="5" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="Z20" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA20" s="9" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="AB20" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC20" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AD20" s="65" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AF20" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH20" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ20" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK20" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL20" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM20" s="8" t="n">
         <v>45612</v>
@@ -22335,7 +22241,7 @@
         <v>158</v>
       </c>
       <c r="AP20" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AR20" s="8"/>
       <c r="AS20" s="8"/>
@@ -22386,10 +22292,10 @@
       <c r="BW20" s="37"/>
       <c r="BX20" s="80"/>
       <c r="BY20" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ20" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA20" s="67" t="n">
         <v>45612</v>
@@ -22398,10 +22304,10 @@
         <v>45613</v>
       </c>
       <c r="CC20" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD20" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE20" s="67" t="n">
         <v>45612</v>
@@ -22410,7 +22316,7 @@
         <v>45613</v>
       </c>
       <c r="CG20" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22442,10 +22348,10 @@
         <v>145</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="M21" s="1" t="s">
         <v>148</v>
@@ -22457,13 +22363,13 @@
         <v>292</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="Q21" s="77" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="R21" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S21" s="9" t="s">
         <v>119</v>
@@ -22475,46 +22381,46 @@
         <v>120</v>
       </c>
       <c r="V21" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W21" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X21" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y21" s="5" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="Z21" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA21" s="9" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="AB21" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC21" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AD21" s="65" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AF21" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH21" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ21" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK21" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL21" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM21" s="8" t="n">
         <v>45612</v>
@@ -22526,7 +22432,7 @@
         <v>158</v>
       </c>
       <c r="AP21" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AR21" s="8"/>
       <c r="AS21" s="8"/>
@@ -22577,10 +22483,10 @@
       <c r="BW21" s="37"/>
       <c r="BX21" s="80"/>
       <c r="BY21" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ21" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA21" s="67" t="n">
         <v>45612</v>
@@ -22589,10 +22495,10 @@
         <v>45613</v>
       </c>
       <c r="CC21" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD21" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE21" s="67" t="n">
         <v>45612</v>
@@ -22601,7 +22507,7 @@
         <v>45613</v>
       </c>
       <c r="CG21" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22633,10 +22539,10 @@
         <v>145</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>148</v>
@@ -22648,13 +22554,13 @@
         <v>333</v>
       </c>
       <c r="P22" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="Q22" s="77" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="R22" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S22" s="9" t="s">
         <v>119</v>
@@ -22666,46 +22572,46 @@
         <v>120</v>
       </c>
       <c r="V22" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W22" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X22" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y22" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z22" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA22" s="9" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="AB22" s="9" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="AC22" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD22" s="65" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="AF22" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH22" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ22" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK22" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL22" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM22" s="8" t="n">
         <v>45612</v>
@@ -22717,7 +22623,7 @@
         <v>158</v>
       </c>
       <c r="AP22" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ22" s="9" t="s">
         <v>135</v>
@@ -22732,7 +22638,7 @@
         <v>158</v>
       </c>
       <c r="AU22" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA22" s="36" t="s">
         <v>141</v>
@@ -22805,7 +22711,7 @@
         <v>0.915972222222222</v>
       </c>
       <c r="BY22" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ22" s="9" t="s">
         <v>143</v>
@@ -22817,7 +22723,7 @@
         <v>45614</v>
       </c>
       <c r="CC22" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD22" s="9" t="s">
         <v>144</v>
@@ -22829,7 +22735,7 @@
         <v>45615</v>
       </c>
       <c r="CG22" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22861,10 +22767,10 @@
         <v>145</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>148</v>
@@ -22876,13 +22782,13 @@
         <v>366</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="Q23" s="77" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="R23" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S23" s="9" t="s">
         <v>119</v>
@@ -22894,46 +22800,46 @@
         <v>120</v>
       </c>
       <c r="V23" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X23" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y23" s="5" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="Z23" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA23" s="9" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="AB23" s="9" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="AC23" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD23" s="65" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="AF23" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH23" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ23" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK23" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL23" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM23" s="8" t="n">
         <v>45612</v>
@@ -22945,7 +22851,7 @@
         <v>158</v>
       </c>
       <c r="AP23" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AR23" s="8"/>
       <c r="AS23" s="8"/>
@@ -23008,7 +22914,7 @@
         <v>45615</v>
       </c>
       <c r="CG23" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23040,10 +22946,10 @@
         <v>145</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>148</v>
@@ -23055,13 +22961,13 @@
         <v>329</v>
       </c>
       <c r="P24" s="9" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="Q24" s="77" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="R24" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S24" s="9" t="s">
         <v>119</v>
@@ -23073,46 +22979,46 @@
         <v>120</v>
       </c>
       <c r="V24" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W24" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X24" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y24" s="5" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="Z24" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA24" s="9" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="AB24" s="9" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="AC24" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD24" s="65" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="AF24" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH24" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ24" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK24" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL24" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM24" s="8" t="n">
         <v>45612</v>
@@ -23124,7 +23030,7 @@
         <v>158</v>
       </c>
       <c r="AP24" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ24" s="9" t="s">
         <v>135</v>
@@ -23139,7 +23045,7 @@
         <v>158</v>
       </c>
       <c r="AU24" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA24" s="36" t="s">
         <v>141</v>
@@ -23212,7 +23118,7 @@
         <v>0.328472222222222</v>
       </c>
       <c r="BY24" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ24" s="9" t="s">
         <v>143</v>
@@ -23224,7 +23130,7 @@
         <v>45614</v>
       </c>
       <c r="CC24" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD24" s="9" t="s">
         <v>144</v>
@@ -23236,7 +23142,7 @@
         <v>45615</v>
       </c>
       <c r="CG24" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23268,10 +23174,10 @@
         <v>145</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="M25" s="1" t="s">
         <v>148</v>
@@ -23283,13 +23189,13 @@
         <v>425</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="Q25" s="77" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="R25" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S25" s="9" t="s">
         <v>119</v>
@@ -23301,46 +23207,46 @@
         <v>120</v>
       </c>
       <c r="V25" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W25" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X25" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y25" s="5" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="Z25" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA25" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="AB25" s="9" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="AC25" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD25" s="65" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="AF25" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH25" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ25" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK25" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL25" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM25" s="8" t="n">
         <v>45612</v>
@@ -23352,7 +23258,7 @@
         <v>158</v>
       </c>
       <c r="AP25" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ25" s="9" t="s">
         <v>135</v>
@@ -23367,7 +23273,7 @@
         <v>158</v>
       </c>
       <c r="AU25" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA25" s="36" t="s">
         <v>141</v>
@@ -23440,7 +23346,7 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY25" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ25" s="9" t="s">
         <v>143</v>
@@ -23452,7 +23358,7 @@
         <v>45614</v>
       </c>
       <c r="CC25" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD25" s="9" t="s">
         <v>144</v>
@@ -23464,7 +23370,7 @@
         <v>45615</v>
       </c>
       <c r="CG25" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23496,10 +23402,10 @@
         <v>145</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>148</v>
@@ -23511,13 +23417,13 @@
         <v>323</v>
       </c>
       <c r="P26" s="9" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="Q26" s="77" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="R26" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S26" s="9" t="s">
         <v>119</v>
@@ -23529,46 +23435,46 @@
         <v>120</v>
       </c>
       <c r="V26" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W26" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X26" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y26" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z26" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="AA26" s="9" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="AB26" s="9" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="AC26" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD26" s="65" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="AF26" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH26" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ26" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK26" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL26" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM26" s="8" t="n">
         <v>45612</v>
@@ -23580,7 +23486,7 @@
         <v>158</v>
       </c>
       <c r="AP26" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ26" s="9" t="s">
         <v>135</v>
@@ -23595,7 +23501,7 @@
         <v>158</v>
       </c>
       <c r="AU26" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA26" s="36" t="s">
         <v>141</v>
@@ -23668,7 +23574,7 @@
         <v>0.915972222222222</v>
       </c>
       <c r="BY26" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ26" s="9" t="s">
         <v>143</v>
@@ -23680,7 +23586,7 @@
         <v>45614</v>
       </c>
       <c r="CC26" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD26" s="9" t="s">
         <v>144</v>
@@ -23692,7 +23598,7 @@
         <v>45615</v>
       </c>
       <c r="CG26" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23724,10 +23630,10 @@
         <v>145</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>148</v>
@@ -23739,64 +23645,64 @@
         <v>255</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="Q27" s="77" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="R27" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S27" s="9" t="s">
         <v>119</v>
       </c>
       <c r="T27" s="9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U27" s="9" t="s">
         <v>120</v>
       </c>
       <c r="V27" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W27" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X27" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y27" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z27" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA27" s="9" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="AB27" s="9" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC27" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD27" s="65" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="AF27" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH27" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ27" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK27" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL27" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM27" s="8" t="n">
         <v>45612</v>
@@ -23808,7 +23714,7 @@
         <v>158</v>
       </c>
       <c r="AP27" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ27" s="9" t="s">
         <v>135</v>
@@ -23823,7 +23729,7 @@
         <v>158</v>
       </c>
       <c r="AU27" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA27" s="36" t="s">
         <v>141</v>
@@ -23908,7 +23814,7 @@
         <v>45615</v>
       </c>
       <c r="CG27" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23940,10 +23846,10 @@
         <v>145</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>148</v>
@@ -23955,13 +23861,13 @@
         <v>337</v>
       </c>
       <c r="P28" s="9" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="Q28" s="77" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="R28" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S28" s="9" t="s">
         <v>119</v>
@@ -23973,46 +23879,46 @@
         <v>120</v>
       </c>
       <c r="V28" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W28" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X28" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y28" s="5" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="Z28" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA28" s="9" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="AB28" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC28" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD28" s="65" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AF28" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH28" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ28" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK28" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL28" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM28" s="8" t="n">
         <v>45612</v>
@@ -24024,7 +23930,7 @@
         <v>158</v>
       </c>
       <c r="AP28" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ28" s="9" t="s">
         <v>135</v>
@@ -24039,7 +23945,7 @@
         <v>158</v>
       </c>
       <c r="AU28" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA28" s="36" t="s">
         <v>141</v>
@@ -24124,7 +24030,7 @@
         <v>45615</v>
       </c>
       <c r="CG28" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24156,10 +24062,10 @@
         <v>145</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="M29" s="1" t="s">
         <v>148</v>
@@ -24171,13 +24077,13 @@
         <v>333</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="Q29" s="77" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="R29" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S29" s="9" t="s">
         <v>119</v>
@@ -24189,46 +24095,46 @@
         <v>120</v>
       </c>
       <c r="V29" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W29" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X29" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y29" s="5" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="Z29" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA29" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AB29" s="9" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="AC29" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD29" s="65" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="AF29" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH29" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ29" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK29" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL29" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM29" s="8" t="n">
         <v>45612</v>
@@ -24240,7 +24146,7 @@
         <v>158</v>
       </c>
       <c r="AP29" s="9" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AQ29" s="9" t="s">
         <v>135</v>
@@ -24255,7 +24161,7 @@
         <v>158</v>
       </c>
       <c r="AU29" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA29" s="36" t="s">
         <v>141</v>
@@ -24328,7 +24234,7 @@
         <v>0.0215277777777778</v>
       </c>
       <c r="BY29" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ29" s="9" t="s">
         <v>143</v>
@@ -24340,7 +24246,7 @@
         <v>45614</v>
       </c>
       <c r="CC29" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="CD29" s="9" t="s">
         <v>144</v>
@@ -24352,7 +24258,7 @@
         <v>45615</v>
       </c>
       <c r="CG29" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24384,10 +24290,10 @@
         <v>145</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="L30" s="9" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="M30" s="1" t="s">
         <v>148</v>
@@ -24396,16 +24302,16 @@
         <v>308</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="P30" s="9" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="Q30" s="77" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="R30" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S30" s="9" t="s">
         <v>119</v>
@@ -24417,46 +24323,46 @@
         <v>120</v>
       </c>
       <c r="V30" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W30" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X30" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y30" s="5" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="Z30" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA30" s="9" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="AB30" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC30" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD30" s="65" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="AF30" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH30" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ30" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK30" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL30" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM30" s="8" t="n">
         <v>45612</v>
@@ -24468,7 +24374,7 @@
         <v>175</v>
       </c>
       <c r="AP30" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ30" s="9" t="s">
         <v>135</v>
@@ -24483,7 +24389,7 @@
         <v>175</v>
       </c>
       <c r="AU30" s="9" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="BA30" s="36" t="s">
         <v>141</v>
@@ -24556,10 +24462,10 @@
         <v>0.5</v>
       </c>
       <c r="BY30" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ30" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA30" s="67" t="n">
         <v>45612</v>
@@ -24568,10 +24474,10 @@
         <v>45613</v>
       </c>
       <c r="CC30" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD30" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE30" s="67" t="n">
         <v>45612</v>
@@ -24580,7 +24486,7 @@
         <v>45613</v>
       </c>
       <c r="CG30" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24612,10 +24518,10 @@
         <v>145</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="M31" s="1" t="s">
         <v>148</v>
@@ -24627,13 +24533,13 @@
         <v>376</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="Q31" s="77" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="R31" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S31" s="9" t="s">
         <v>119</v>
@@ -24645,46 +24551,46 @@
         <v>120</v>
       </c>
       <c r="V31" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W31" s="8" t="n">
         <v>45614</v>
       </c>
       <c r="X31" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="Y31" s="5" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="Z31" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AA31" s="9" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="AB31" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC31" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="AD31" s="65" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="AF31" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH31" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ31" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK31" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL31" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM31" s="8" t="n">
         <v>45612</v>
@@ -24696,7 +24602,7 @@
         <v>158</v>
       </c>
       <c r="AP31" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AQ31" s="9" t="s">
         <v>135</v>
@@ -24711,7 +24617,7 @@
         <v>158</v>
       </c>
       <c r="AU31" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA31" s="36" t="s">
         <v>141</v>
@@ -24784,10 +24690,10 @@
         <v>0.5</v>
       </c>
       <c r="BY31" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="BZ31" s="9" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="CA31" s="67" t="n">
         <v>45612</v>
@@ -24796,10 +24702,10 @@
         <v>45613</v>
       </c>
       <c r="CC31" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="CD31" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="CE31" s="67" t="n">
         <v>45612</v>
@@ -24808,7 +24714,7 @@
         <v>45613</v>
       </c>
       <c r="CG31" s="9" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="32" s="51" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24841,10 +24747,10 @@
         <v>145</v>
       </c>
       <c r="K32" s="51" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="L32" s="51" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="M32" s="42" t="s">
         <v>148</v>
@@ -24856,59 +24762,59 @@
         <v>360</v>
       </c>
       <c r="P32" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="Q32" s="83" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="R32" s="51" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S32" s="51" t="s">
         <v>119</v>
       </c>
       <c r="T32" s="51" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="U32" s="51" t="s">
         <v>120</v>
       </c>
       <c r="V32" s="51" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W32" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X32" s="51" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y32" s="84" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="Z32" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA32" s="51" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="AB32" s="51" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AC32" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD32" s="85" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AE32" s="86"/>
       <c r="AF32" s="87" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH32" s="84" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ32" s="51" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK32" s="88" t="n">
         <v>3</v>
@@ -24983,10 +24889,10 @@
         <v>145</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="L33" s="9" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>148</v>
@@ -24998,13 +24904,13 @@
         <v>209</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="Q33" s="77" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="R33" s="9" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="S33" s="9" t="s">
         <v>119</v>
@@ -25016,46 +24922,46 @@
         <v>120</v>
       </c>
       <c r="V33" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="W33" s="8" t="n">
         <v>45615</v>
       </c>
       <c r="X33" s="9" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="Y33" s="5" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="Z33" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AA33" s="9" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="AB33" s="9" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AC33" s="8" t="n">
         <v>45616</v>
       </c>
       <c r="AD33" s="65" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AF33" s="38" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AH33" s="5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AJ33" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AK33" s="2" t="n">
         <v>3</v>
       </c>
       <c r="AL33" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM33" s="8" t="n">
         <v>45612</v>
@@ -25067,7 +24973,7 @@
         <v>158</v>
       </c>
       <c r="AP33" s="9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AQ33" s="9" t="s">
         <v>135</v>
@@ -25082,7 +24988,7 @@
         <v>158</v>
       </c>
       <c r="AU33" s="9" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="BA33" s="36" t="s">
         <v>141</v>
@@ -25155,7 +25061,7 @@
         <v>0.474305555555556</v>
       </c>
       <c r="BY33" s="1" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="BZ33" s="9" t="s">
         <v>144</v>
@@ -25167,7 +25073,7 @@
         <v>45616</v>
       </c>
       <c r="CC33" s="9" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="34" s="51" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25200,10 +25106,10 @@
         <v>145</v>
       </c>
       <c r="K34" s="51" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="L34" s="51" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="M34" s="42" t="s">
         <v>148</v>
@@ -25215,10 +25121,10 @@
         <v>383</v>
       </c>
       <c r="P34" s="51" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="Q34" s="83" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="R34" s="51" t="s">
         <v>120</v>
@@ -25308,10 +25214,10 @@
         <v>145</v>
       </c>
       <c r="K35" s="51" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="L35" s="51" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="M35" s="42" t="s">
         <v>114</v>
@@ -25323,10 +25229,10 @@
         <v>209</v>
       </c>
       <c r="P35" s="51" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="Q35" s="83" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="R35" s="51" t="s">
         <v>120</v>
@@ -25416,10 +25322,10 @@
         <v>145</v>
       </c>
       <c r="K36" s="51" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="L36" s="51" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="M36" s="42" t="s">
         <v>148</v>
@@ -25431,10 +25337,10 @@
         <v>226</v>
       </c>
       <c r="P36" s="51" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="Q36" s="83" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="R36" s="51" t="s">
         <v>120</v>
@@ -25525,10 +25431,10 @@
         <v>145</v>
       </c>
       <c r="K37" s="51" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="L37" s="51" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="M37" s="42" t="s">
         <v>148</v>
@@ -25540,10 +25446,10 @@
         <v>149</v>
       </c>
       <c r="P37" s="51" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="Q37" s="83" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="R37" s="51" t="s">
         <v>120</v>

</xml_diff>

<commit_message>
Asisgnacion de viaje en proceso. Asignacion de tripulante, buque y eta.
</commit_message>
<xml_diff>
--- a/Carga_Real.xlsx
+++ b/Carga_Real.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" state="visible" r:id="rId3"/>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">Vessel </t>
+    <t xml:space="preserve">Vessel</t>
   </si>
   <si>
     <t xml:space="preserve">Date arrive CL</t>

</xml_diff>